<commit_message>
Update Sprint BackLog for Sprint 2 with new changes
</commit_message>
<xml_diff>
--- a/sprint backlog/Sprint BackLog Sprint2.xlsx
+++ b/sprint backlog/Sprint BackLog Sprint2.xlsx
@@ -5,19 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Software Engineering\PaiNamNaeWebAppSec2_6\sprint backlog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E1CF4E54-0778-471E-B52D-6C275050853E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{869B4A08-0261-4005-A252-220B1ADD8712}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -36,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="55">
   <si>
     <t>SPRINT 2 BACKLOG</t>
   </si>
@@ -135,9 +132,6 @@
   </si>
   <si>
     <t>วงศ์ปกรณ์</t>
-  </si>
-  <si>
-    <t>In-progress</t>
   </si>
   <si>
     <t>เขียน API Testing</t>
@@ -549,22 +543,6 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -575,15 +553,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -592,6 +561,31 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1689,131 +1683,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="SprintBacklog"/>
-      <sheetName val="Sheet1"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="6">
-          <cell r="U6" t="str">
-            <v>Total Remaining Effort</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="U8">
-            <v>40</v>
-          </cell>
-          <cell r="V8">
-            <v>40</v>
-          </cell>
-          <cell r="W8">
-            <v>38</v>
-          </cell>
-          <cell r="X8">
-            <v>38</v>
-          </cell>
-          <cell r="Y8">
-            <v>25</v>
-          </cell>
-          <cell r="Z8">
-            <v>25</v>
-          </cell>
-          <cell r="AA8">
-            <v>25</v>
-          </cell>
-          <cell r="AB8">
-            <v>4</v>
-          </cell>
-          <cell r="AC8">
-            <v>4</v>
-          </cell>
-          <cell r="AD8">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="T13" t="str">
-            <v>Ideal Remaining Effort</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="U14">
-            <v>1</v>
-          </cell>
-          <cell r="V14">
-            <v>2</v>
-          </cell>
-          <cell r="W14">
-            <v>3</v>
-          </cell>
-          <cell r="X14">
-            <v>4</v>
-          </cell>
-          <cell r="Y14">
-            <v>5</v>
-          </cell>
-          <cell r="Z14">
-            <v>6</v>
-          </cell>
-          <cell r="AA14">
-            <v>7</v>
-          </cell>
-          <cell r="AB14">
-            <v>8</v>
-          </cell>
-          <cell r="AC14">
-            <v>9</v>
-          </cell>
-          <cell r="AD14">
-            <v>10</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="U15">
-            <v>36</v>
-          </cell>
-          <cell r="V15">
-            <v>32</v>
-          </cell>
-          <cell r="W15">
-            <v>28</v>
-          </cell>
-          <cell r="X15">
-            <v>24</v>
-          </cell>
-          <cell r="Y15">
-            <v>20</v>
-          </cell>
-          <cell r="Z15">
-            <v>16</v>
-          </cell>
-          <cell r="AA15">
-            <v>12</v>
-          </cell>
-          <cell r="AB15">
-            <v>8</v>
-          </cell>
-          <cell r="AC15">
-            <v>4</v>
-          </cell>
-          <cell r="AD15">
-            <v>0</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
@@ -2027,21 +1896,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="11"/>
+      <c r="A1" s="25" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="21"/>
     </row>
     <row r="2" spans="1:25" ht="21.6" x14ac:dyDescent="0.4">
       <c r="A2" s="2"/>
@@ -2057,16 +1926,16 @@
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
-      <c r="R2" s="15" t="s">
+      <c r="R2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="S2" s="10"/>
-      <c r="T2" s="10"/>
-      <c r="U2" s="10"/>
-      <c r="V2" s="10"/>
-      <c r="W2" s="10"/>
-      <c r="X2" s="10"/>
-      <c r="Y2" s="11"/>
+      <c r="S2" s="20"/>
+      <c r="T2" s="20"/>
+      <c r="U2" s="20"/>
+      <c r="V2" s="20"/>
+      <c r="W2" s="20"/>
+      <c r="X2" s="20"/>
+      <c r="Y2" s="21"/>
     </row>
     <row r="3" spans="1:25" ht="33.6" x14ac:dyDescent="0.75">
       <c r="A3" s="3" t="s">
@@ -2108,7 +1977,7 @@
       <c r="M3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="N3" s="17" t="s">
+      <c r="N3" s="9" t="s">
         <v>15</v>
       </c>
       <c r="R3" s="4" t="s">
@@ -2137,10 +2006,10 @@
       </c>
     </row>
     <row r="4" spans="1:25" ht="30" x14ac:dyDescent="0.85">
-      <c r="A4" s="12">
+      <c r="A4" s="26">
         <v>1</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="26" t="s">
         <v>17</v>
       </c>
       <c r="C4" s="6" t="s">
@@ -2180,41 +2049,41 @@
         <f>SUM(F4:F29)</f>
         <v>74</v>
       </c>
-      <c r="R4" s="25" t="s">
-        <v>55</v>
-      </c>
-      <c r="S4" s="26">
+      <c r="R4" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="S4" s="15">
         <f>G30</f>
         <v>67</v>
       </c>
-      <c r="T4" s="26">
-        <f t="shared" ref="S4:Y4" si="0">H30</f>
+      <c r="T4" s="15">
+        <f t="shared" ref="T4:Y4" si="0">H30</f>
         <v>52</v>
       </c>
-      <c r="U4" s="26">
+      <c r="U4" s="15">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="V4" s="26">
+      <c r="V4" s="15">
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
-      <c r="W4" s="26">
+      <c r="W4" s="15">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="X4" s="26">
+      <c r="X4" s="15">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="Y4" s="26">
+      <c r="Y4" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:25" ht="63.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="13"/>
-      <c r="B5" s="13"/>
+      <c r="A5" s="17"/>
+      <c r="B5" s="17"/>
       <c r="C5" s="6" t="s">
         <v>21</v>
       </c>
@@ -2248,11 +2117,11 @@
       <c r="M5" s="7">
         <v>0</v>
       </c>
-      <c r="N5" s="13"/>
+      <c r="N5" s="17"/>
     </row>
     <row r="6" spans="1:25" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
-      <c r="A6" s="13"/>
-      <c r="B6" s="13"/>
+      <c r="A6" s="17"/>
+      <c r="B6" s="17"/>
       <c r="C6" s="6" t="s">
         <v>23</v>
       </c>
@@ -2286,21 +2155,21 @@
       <c r="M6" s="7">
         <v>0</v>
       </c>
-      <c r="N6" s="13"/>
-      <c r="R6" s="23" t="s">
-        <v>54</v>
-      </c>
-      <c r="S6" s="21"/>
-      <c r="T6" s="21"/>
-      <c r="U6" s="21"/>
-      <c r="V6" s="21"/>
-      <c r="W6" s="21"/>
-      <c r="X6" s="21"/>
-      <c r="Y6" s="22"/>
+      <c r="N6" s="17"/>
+      <c r="R6" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="S6" s="23"/>
+      <c r="T6" s="23"/>
+      <c r="U6" s="23"/>
+      <c r="V6" s="23"/>
+      <c r="W6" s="23"/>
+      <c r="X6" s="23"/>
+      <c r="Y6" s="24"/>
     </row>
     <row r="7" spans="1:25" ht="53.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.8">
-      <c r="A7" s="13"/>
-      <c r="B7" s="13"/>
+      <c r="A7" s="17"/>
+      <c r="B7" s="17"/>
       <c r="C7" s="6" t="s">
         <v>25</v>
       </c>
@@ -2334,35 +2203,35 @@
       <c r="M7" s="7">
         <v>0</v>
       </c>
-      <c r="N7" s="13"/>
-      <c r="R7" s="19" t="s">
+      <c r="N7" s="17"/>
+      <c r="R7" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="S7" s="20">
+      <c r="S7" s="12">
         <v>1</v>
       </c>
-      <c r="T7" s="20">
-        <v>2</v>
-      </c>
-      <c r="U7" s="20">
+      <c r="T7" s="12">
+        <v>2</v>
+      </c>
+      <c r="U7" s="12">
         <v>3</v>
       </c>
-      <c r="V7" s="20">
+      <c r="V7" s="12">
         <v>4</v>
       </c>
-      <c r="W7" s="20">
+      <c r="W7" s="12">
         <v>5</v>
       </c>
-      <c r="X7" s="20">
+      <c r="X7" s="12">
         <v>6</v>
       </c>
-      <c r="Y7" s="20">
+      <c r="Y7" s="12">
         <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:25" ht="108" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A8" s="13"/>
-      <c r="B8" s="13"/>
+      <c r="A8" s="17"/>
+      <c r="B8" s="17"/>
       <c r="C8" s="6" t="s">
         <v>27</v>
       </c>
@@ -2396,42 +2265,42 @@
       <c r="M8" s="7">
         <v>0</v>
       </c>
-      <c r="N8" s="13"/>
-      <c r="R8" s="18" t="s">
-        <v>55</v>
-      </c>
-      <c r="S8" s="24">
+      <c r="N8" s="17"/>
+      <c r="R8" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="S8" s="13">
         <f>N4-N4/7*1</f>
         <v>63.428571428571431</v>
       </c>
-      <c r="T8" s="24">
+      <c r="T8" s="13">
         <f>N4-N4/7*2</f>
         <v>52.857142857142861</v>
       </c>
-      <c r="U8" s="24">
+      <c r="U8" s="13">
         <f>N4-N4/7*3</f>
         <v>42.285714285714285</v>
       </c>
-      <c r="V8" s="24">
+      <c r="V8" s="13">
         <f>N4-N4/7*4</f>
         <v>31.714285714285715</v>
       </c>
-      <c r="W8" s="24">
+      <c r="W8" s="13">
         <f>N4-N4/7*5</f>
         <v>21.142857142857146</v>
       </c>
-      <c r="X8" s="24">
+      <c r="X8" s="13">
         <f>N4-N4/7*6</f>
         <v>10.571428571428569</v>
       </c>
-      <c r="Y8" s="24">
+      <c r="Y8" s="13">
         <f>N4-N4/7*7</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:25" ht="69" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="13"/>
-      <c r="B9" s="13"/>
+      <c r="A9" s="17"/>
+      <c r="B9" s="17"/>
       <c r="C9" s="6" t="s">
         <v>28</v>
       </c>
@@ -2465,11 +2334,11 @@
       <c r="M9" s="7">
         <v>0</v>
       </c>
-      <c r="N9" s="13"/>
+      <c r="N9" s="17"/>
     </row>
     <row r="10" spans="1:25" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="13"/>
-      <c r="B10" s="13"/>
+      <c r="A10" s="17"/>
+      <c r="B10" s="17"/>
       <c r="C10" s="6" t="s">
         <v>29</v>
       </c>
@@ -2503,11 +2372,11 @@
       <c r="M10" s="7">
         <v>0</v>
       </c>
-      <c r="N10" s="13"/>
+      <c r="N10" s="17"/>
     </row>
     <row r="11" spans="1:25" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="13"/>
-      <c r="B11" s="13"/>
+      <c r="A11" s="17"/>
+      <c r="B11" s="17"/>
       <c r="C11" s="6" t="s">
         <v>30</v>
       </c>
@@ -2541,11 +2410,11 @@
       <c r="M11" s="7">
         <v>0</v>
       </c>
-      <c r="N11" s="13"/>
+      <c r="N11" s="17"/>
     </row>
     <row r="12" spans="1:25" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="13"/>
-      <c r="B12" s="13"/>
+      <c r="A12" s="17"/>
+      <c r="B12" s="17"/>
       <c r="C12" s="6" t="s">
         <v>31</v>
       </c>
@@ -2553,7 +2422,7 @@
         <v>32</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="F12" s="7">
         <v>5</v>
@@ -2579,13 +2448,13 @@
       <c r="M12" s="7">
         <v>0</v>
       </c>
-      <c r="N12" s="13"/>
+      <c r="N12" s="17"/>
     </row>
     <row r="13" spans="1:25" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="13"/>
-      <c r="B13" s="13"/>
+      <c r="A13" s="17"/>
+      <c r="B13" s="17"/>
       <c r="C13" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>22</v>
@@ -2617,19 +2486,19 @@
       <c r="M13" s="7">
         <v>0</v>
       </c>
-      <c r="N13" s="13"/>
+      <c r="N13" s="17"/>
     </row>
     <row r="14" spans="1:25" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="13"/>
-      <c r="B14" s="13"/>
+      <c r="A14" s="17"/>
+      <c r="B14" s="17"/>
       <c r="C14" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>32</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="F14" s="7"/>
       <c r="G14" s="7"/>
@@ -2639,19 +2508,19 @@
       <c r="K14" s="7"/>
       <c r="L14" s="7"/>
       <c r="M14" s="7"/>
-      <c r="N14" s="13"/>
+      <c r="N14" s="17"/>
     </row>
     <row r="15" spans="1:25" ht="99.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="14"/>
-      <c r="B15" s="14"/>
+      <c r="A15" s="18"/>
+      <c r="B15" s="18"/>
       <c r="C15" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>22</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="F15" s="7">
         <v>1</v>
@@ -2677,14 +2546,14 @@
       <c r="M15" s="7">
         <v>0</v>
       </c>
-      <c r="N15" s="13"/>
+      <c r="N15" s="17"/>
     </row>
     <row r="16" spans="1:25" ht="69" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="12">
+      <c r="A16" s="26">
         <v>16</v>
       </c>
-      <c r="B16" s="12" t="s">
-        <v>37</v>
+      <c r="B16" s="26" t="s">
+        <v>36</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>18</v>
@@ -2719,13 +2588,13 @@
       <c r="M16" s="7">
         <v>0</v>
       </c>
-      <c r="N16" s="13"/>
+      <c r="N16" s="17"/>
     </row>
     <row r="17" spans="1:14" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="13"/>
-      <c r="B17" s="13"/>
+      <c r="A17" s="17"/>
+      <c r="B17" s="17"/>
       <c r="C17" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>26</v>
@@ -2757,13 +2626,13 @@
       <c r="M17" s="7">
         <v>0</v>
       </c>
-      <c r="N17" s="13"/>
+      <c r="N17" s="17"/>
     </row>
     <row r="18" spans="1:14" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="13"/>
-      <c r="B18" s="13"/>
+      <c r="A18" s="17"/>
+      <c r="B18" s="17"/>
       <c r="C18" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>26</v>
@@ -2795,16 +2664,16 @@
       <c r="M18" s="7">
         <v>0</v>
       </c>
-      <c r="N18" s="13"/>
+      <c r="N18" s="17"/>
     </row>
     <row r="19" spans="1:14" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="13"/>
-      <c r="B19" s="13"/>
+      <c r="A19" s="17"/>
+      <c r="B19" s="17"/>
       <c r="C19" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>20</v>
@@ -2833,16 +2702,16 @@
       <c r="M19" s="7">
         <v>0</v>
       </c>
-      <c r="N19" s="13"/>
+      <c r="N19" s="17"/>
     </row>
     <row r="20" spans="1:14" ht="55.2" x14ac:dyDescent="0.25">
-      <c r="A20" s="13"/>
-      <c r="B20" s="13"/>
+      <c r="A20" s="17"/>
+      <c r="B20" s="17"/>
       <c r="C20" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E20" s="7" t="s">
         <v>20</v>
@@ -2871,13 +2740,13 @@
       <c r="M20" s="7">
         <v>0</v>
       </c>
-      <c r="N20" s="13"/>
+      <c r="N20" s="17"/>
     </row>
     <row r="21" spans="1:14" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="A21" s="13"/>
-      <c r="B21" s="13"/>
+      <c r="A21" s="17"/>
+      <c r="B21" s="17"/>
       <c r="C21" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>24</v>
@@ -2909,19 +2778,19 @@
       <c r="M21" s="7">
         <v>0</v>
       </c>
-      <c r="N21" s="13"/>
+      <c r="N21" s="17"/>
     </row>
     <row r="22" spans="1:14" ht="55.2" x14ac:dyDescent="0.25">
-      <c r="A22" s="13"/>
-      <c r="B22" s="13"/>
+      <c r="A22" s="17"/>
+      <c r="B22" s="17"/>
       <c r="C22" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D22" s="7" t="s">
-        <v>45</v>
-      </c>
       <c r="E22" s="7" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="F22" s="7">
         <v>6</v>
@@ -2947,19 +2816,19 @@
       <c r="M22" s="7">
         <v>0</v>
       </c>
-      <c r="N22" s="13"/>
+      <c r="N22" s="17"/>
     </row>
     <row r="23" spans="1:14" ht="82.8" x14ac:dyDescent="0.25">
-      <c r="A23" s="13"/>
-      <c r="B23" s="13"/>
+      <c r="A23" s="17"/>
+      <c r="B23" s="17"/>
       <c r="C23" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="F23" s="7">
         <v>6</v>
@@ -2985,13 +2854,13 @@
       <c r="M23" s="7">
         <v>0</v>
       </c>
-      <c r="N23" s="13"/>
+      <c r="N23" s="17"/>
     </row>
     <row r="24" spans="1:14" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="13"/>
-      <c r="B24" s="13"/>
+      <c r="A24" s="17"/>
+      <c r="B24" s="17"/>
       <c r="C24" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D24" s="7" t="s">
         <v>32</v>
@@ -3023,13 +2892,13 @@
       <c r="M24" s="7">
         <v>0</v>
       </c>
-      <c r="N24" s="13"/>
+      <c r="N24" s="17"/>
     </row>
     <row r="25" spans="1:14" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="13"/>
-      <c r="B25" s="13"/>
+      <c r="A25" s="17"/>
+      <c r="B25" s="17"/>
       <c r="C25" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D25" s="7" t="s">
         <v>22</v>
@@ -3061,13 +2930,13 @@
       <c r="M25" s="7">
         <v>0</v>
       </c>
-      <c r="N25" s="13"/>
+      <c r="N25" s="17"/>
     </row>
     <row r="26" spans="1:14" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="13"/>
-      <c r="B26" s="13"/>
+      <c r="A26" s="17"/>
+      <c r="B26" s="17"/>
       <c r="C26" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>22</v>
@@ -3099,13 +2968,13 @@
       <c r="M26" s="7">
         <v>0</v>
       </c>
-      <c r="N26" s="13"/>
+      <c r="N26" s="17"/>
     </row>
     <row r="27" spans="1:14" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="13"/>
-      <c r="B27" s="13"/>
+      <c r="A27" s="17"/>
+      <c r="B27" s="17"/>
       <c r="C27" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D27" s="7" t="s">
         <v>32</v>
@@ -3133,19 +3002,19 @@
       <c r="M27" s="7">
         <v>0</v>
       </c>
-      <c r="N27" s="13"/>
+      <c r="N27" s="17"/>
     </row>
     <row r="28" spans="1:14" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="13"/>
-      <c r="B28" s="13"/>
+      <c r="A28" s="17"/>
+      <c r="B28" s="17"/>
       <c r="C28" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="F28" s="7">
         <v>2</v>
@@ -3171,19 +3040,19 @@
       <c r="M28" s="7">
         <v>0</v>
       </c>
-      <c r="N28" s="13"/>
+      <c r="N28" s="17"/>
     </row>
     <row r="29" spans="1:14" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="14"/>
-      <c r="B29" s="14"/>
+      <c r="A29" s="18"/>
+      <c r="B29" s="18"/>
       <c r="C29" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D29" s="7" t="s">
         <v>19</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="F29" s="7">
         <v>2</v>
@@ -3209,11 +3078,11 @@
       <c r="M29" s="7">
         <v>0</v>
       </c>
-      <c r="N29" s="14"/>
+      <c r="N29" s="18"/>
     </row>
     <row r="30" spans="1:14" ht="13.2" x14ac:dyDescent="0.25">
       <c r="E30" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F30" s="8">
         <f t="shared" ref="F30:M30" si="1">SUM(F4:F29)</f>

</xml_diff>